<commit_message>
Audit and stabilize domain task surfaces
</commit_message>
<xml_diff>
--- a/task-reviews/geometry/task_geometry_analytical_3d_value/task_geometry_analytical_3d_value.xlsx
+++ b/task-reviews/geometry/task_geometry_analytical_3d_value/task_geometry_analytical_3d_value.xlsx
@@ -3029,36 +3029,36 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Look at the annotated image showing an annotated 3D solid. Based on the shown values, answer this question: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
+          <t>The image shows an annotated 3D solid. Question: The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: KL, ML.
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"KL":2,"ML":3},"answer":"12π"}</t>
+Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: CD, EF.
+Answer requirement: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"CD":2,"EF":3},"answer":8}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Look at the annotated image showing an annotated 3D solid. Based on the shown values, answer this question: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
+          <t>The image shows an annotated 3D solid. Question: The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
 Return a valid JSON object with key "answer".
-Answer: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer requirement: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"KL": 11, "ML": 48}, "answer": "649π"}</t>
+          <t>{"evidence": {"CD": 48, "EF": 49}, "answer": 7008}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>{"KL": 11, "ML": 48}</t>
+          <t>{"CD": 48, "EF": 49}</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -3067,16 +3067,16 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>324021735868198</v>
+        <v>585016520816098</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0013.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0012.png</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0013.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0012.json</t>
         </is>
       </c>
     </row>
@@ -3093,17 +3093,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
+          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: HI, JK.
-Answer: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"HI":2,"JK":3},"answer":"12π"}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: IJ, KL.
+Answer field: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"IJ":2,"KL":3},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
+          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
@@ -3112,12 +3112,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"HI": 17, "JK": 15}, "answer": "1088π"}</t>
+          <t>{"evidence": {"IJ": 6, "KL": 44}, "answer": "600π"}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>{"HI": 17, "JK": 15}</t>
+          <t>{"IJ": 6, "KL": 44}</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -3131,16 +3131,16 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>639963341038727</v>
+        <v>834822902431278</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0005.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0013.png</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0005.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0013.json</t>
         </is>
       </c>
     </row>
@@ -3157,31 +3157,31 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Question: The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
+          <t>Look at the annotated image showing an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: IJ, KL.
-Answer format: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"IJ":2,"KL":3},"answer":8}</t>
+Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: KL, LM, KN.
+Answer requirement: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"KL":2,"LM":3,"KN":4},"answer":8}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Question: The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
+          <t>Look at the annotated image showing an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
 Return a valid JSON object with key "answer".
-Answer: set "answer" to the value as an integer.
+Answer field: set "answer" to the value as an integer.
 Example JSON:
 {"answer":8}</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"IJ": 16, "KL": 41}, "answer": 1568}</t>
+          <t>{"evidence": {"KL": 13, "LM": 49, "KN": 23}, "answer": 4126}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>{"IJ": 16, "KL": 41}</t>
+          <t>{"KL": 13, "LM": 49, "KN": 23}</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -3195,16 +3195,16 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>963278194846610</v>
+        <v>1675645771519581</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0002.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0015.png</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0002.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0015.json</t>
         </is>
       </c>
     </row>
@@ -3221,31 +3221,31 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+          <t>You are given an image showing an annotated 3D solid. Task: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: IJ.
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"IJ":2},"answer":"12π"}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: BC, DC.
+Answer field: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"BC":2,"DC":3},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+          <t>You are given an image showing an annotated 3D solid. Task: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer: set "answer" to the value in the form kπ (for example 12π).
+Answer field: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
 {"answer":"12π"}</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"IJ": 7}, "answer": "196π"}</t>
+          <t>{"evidence": {"BC": 36, "DC": 46}, "answer": "2952π"}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>{"IJ": 7}</t>
+          <t>{"BC": 36, "DC": 46}</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -3259,16 +3259,16 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>979734125544075</v>
+        <v>2961404657033117</v>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0024.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0003.png</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0024.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0003.json</t>
         </is>
       </c>
     </row>
@@ -3285,31 +3285,31 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Based on the shown values, answer this question: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: HI, JK.
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"HI":2,"JK":3},"answer":"12π"}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: MN.
+Answer field: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"MN":2},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Based on the shown values, answer this question: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
+Answer: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
 {"answer":"12π"}</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"HI": 49, "JK": 32}, "answer": "7938π"}</t>
+          <t>{"evidence": {"MN": 33}, "answer": "4356π"}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>{"HI": 49, "JK": 32}</t>
+          <t>{"MN": 33}</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -3323,16 +3323,16 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>998055751459479</v>
+        <v>3081582893562271</v>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0022.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0006.png</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0022.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0006.json</t>
         </is>
       </c>
     </row>
@@ -3349,17 +3349,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
+          <t>You are given an image showing an annotated 3D solid. Task: The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: HI, JK.
-Answer format: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"HI":2,"JK":3},"answer":8}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: EF, GH.
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"EF":2,"GH":3},"answer":8}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
+          <t>You are given an image showing an annotated 3D solid. Task: The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
 Return a valid JSON object with key "answer".
 Answer: set "answer" to the value as an integer.
 Example JSON:
@@ -3368,12 +3368,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"HI": 44, "JK": 45}, "answer": 5896}</t>
+          <t>{"evidence": {"EF": 36, "GH": 24}, "answer": 3024}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>{"HI": 44, "JK": 45}</t>
+          <t>{"EF": 36, "GH": 24}</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -3387,16 +3387,16 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>1680120588651168</v>
+        <v>3135267092585094</v>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0023.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0000.png</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0023.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0000.json</t>
         </is>
       </c>
     </row>
@@ -3413,17 +3413,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Question: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: AB.
-Answer: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"AB":2},"answer":"12π"}</t>
+Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: HI.
+Answer requirement: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"HI":2},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Question: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
@@ -3432,12 +3432,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"AB": 32}, "answer": "4096π"}</t>
+          <t>{"evidence": {"HI": 40}, "answer": "6400π"}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>{"AB": 32}</t>
+          <t>{"HI": 40}</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -3451,16 +3451,16 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>2749742435116051</v>
+        <v>4764341336182129</v>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0020.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0001.png</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0020.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0001.json</t>
         </is>
       </c>
     </row>
@@ -3477,31 +3477,31 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Based on the shown values, answer this question: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+          <t>You are given an image showing an annotated 3D solid. Task: The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: GH.
+Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: RS, TU.
 Answer format: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
-{"evidence":{"GH":2},"answer":"12π"}</t>
+{"evidence":{"RS":2,"TU":3},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Based on the shown values, answer this question: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+          <t>You are given an image showing an annotated 3D solid. Task: The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer: set "answer" to the value in the form kπ (for example 12π).
+Answer field: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
 {"answer":"12π"}</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"GH": 49}, "answer": "9604π"}</t>
+          <t>{"evidence": {"RS": 41, "TU": 50}, "answer": "7462π"}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>{"GH": 49}</t>
+          <t>{"RS": 41, "TU": 50}</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -3515,16 +3515,16 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>3040711640956035</v>
+        <v>4983387212272678</v>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0008.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0002.png</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0008.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0002.json</t>
         </is>
       </c>
     </row>
@@ -3541,31 +3541,31 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: LM.
-Answer format: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"LM":2},"answer":"12π"}</t>
+Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: GH, IH.
+Answer rule: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"GH":2,"IH":3},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer: set "answer" to the value in the form kπ (for example 12π).
+Answer rule: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
 {"answer":"12π"}</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"LM": 30}, "answer": "3600π"}</t>
+          <t>{"evidence": {"GH": 11, "IH": 47}, "answer": "638π"}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>{"LM": 30}</t>
+          <t>{"GH": 11, "IH": 47}</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -3579,16 +3579,16 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>3078835629021186</v>
+        <v>5131989709445648</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0015.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0007.png</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0015.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0007.json</t>
         </is>
       </c>
     </row>
@@ -3605,36 +3605,36 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. Task: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Question: The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: OP.
-Answer: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"OP":2},"answer":"12π"}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: UV, WX.
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"UV":2,"WX":3},"answer":8}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. Task: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Question: The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
 Return a valid JSON object with key "answer".
-Answer field: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"OP": 16}, "answer": "1024π"}</t>
+          <t>{"evidence": {"UV": 12, "WX": 30}, "answer": 864}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>{"OP": 16}</t>
+          <t>{"UV": 12, "WX": 30}</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -3643,16 +3643,16 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>4170857945503611</v>
+        <v>5161299296996229</v>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0003.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0021.png</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0003.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0021.json</t>
         </is>
       </c>
     </row>
@@ -3669,31 +3669,31 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Read the marked measurements and answer: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
+          <t>Look at the annotated image showing an annotated 3D solid. Based on the shown values, answer this question: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: NO, OP, NQ.
-Answer requirement: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"NO":2,"OP":3,"NQ":4},"answer":8}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: NO, NP, OP, NQ.
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"NO":2,"NP":3,"OP":4,"NQ":5},"answer":8}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Read the marked measurements and answer: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
+          <t>Look at the annotated image showing an annotated 3D solid. Based on the shown values, answer this question: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
 Return a valid JSON object with key "answer".
-Answer: set "answer" to the value as an integer.
+Answer format: set "answer" to the value as an integer.
 Example JSON:
 {"answer":8}</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"NO": 45, "OP": 5, "NQ": 25}, "answer": 2950}</t>
+          <t>{"evidence": {"NO": 16, "NP": 30, "OP": 34, "NQ": 50}, "answer": 4480}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>{"NO": 45, "OP": 5, "NQ": 25}</t>
+          <t>{"NO": 16, "NP": 30, "OP": 34, "NQ": 50}</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -3707,16 +3707,16 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>4210398867811178</v>
+        <v>5359586476846093</v>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0016.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0019.png</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0016.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0019.json</t>
         </is>
       </c>
     </row>
@@ -3733,17 +3733,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. Question: The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
+          <t>Look at the annotated image showing an annotated 3D solid. Read the marked measurements and answer: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: VW, XY.
+Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: YZ.
 Answer format: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
-{"evidence":{"VW":2,"XY":3},"answer":"12π"}</t>
+{"evidence":{"YZ":2},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. Question: The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
+          <t>Look at the annotated image showing an annotated 3D solid. Read the marked measurements and answer: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
@@ -3752,12 +3752,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"VW": 8, "XY": 43}, "answer": "816π"}</t>
+          <t>{"evidence": {"YZ": 11}, "answer": "484π"}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>{"VW": 8, "XY": 43}</t>
+          <t>{"YZ": 11}</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -3771,16 +3771,16 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>4354268436115484</v>
+        <v>6154022488823990</v>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0017.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0024.png</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0017.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0024.json</t>
         </is>
       </c>
     </row>
@@ -3797,36 +3797,36 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Based on the shown values, answer this question: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
+          <t>You are given an image showing an annotated 3D solid. Question: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: AB, AC, BC, AD.
-Answer field: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"AB":2,"AC":3,"BC":4,"AD":5},"answer":8}</t>
+Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: KL, ML.
+Answer: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"KL":2,"ML":3},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Based on the shown values, answer this question: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
+          <t>You are given an image showing an annotated 3D solid. Question: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer: set "answer" to the value as an integer.
-Example JSON:
-{"answer":8}</t>
+Answer field: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"answer":"12π"}</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"AB": 16, "AC": 30, "BC": 34, "AD": 13}, "answer": 1520}</t>
+          <t>{"evidence": {"KL": 46, "ML": 50}, "answer": "4416π"}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>{"AB": 16, "AC": 30, "BC": 34, "AD": 13}</t>
+          <t>{"KL": 46, "ML": 50}</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>pi_expression</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -3835,16 +3835,16 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>4495639611516914</v>
+        <v>6315476458303255</v>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0012.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0018.png</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0012.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0018.json</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,583 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
+          <t>Use the image showing an annotated 3D solid. The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
+Return a valid JSON object with keys "evidence" and "answer" in that order.
+Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: CD, EF.
+Answer rule: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"CD":2,"EF":3},"answer":8}</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Use the image showing an annotated 3D solid. The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
+Return a valid JSON object with key "answer".
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>{"evidence": {"CD": 14, "EF": 41}, "answer": 1344}</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>{"CD": 14, "EF": 41}</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>measurement_ref_map</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>6317894895206288</v>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0004.png</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0004.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="288" customHeight="1">
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>task_geometry_analytical_3d_value</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>surface_area</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Work from the annotated figure showing an annotated 3D solid. Based on the shown values, answer this question: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+Return a valid JSON object with keys "evidence" and "answer" in that order.
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: MN.
+Answer field: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"MN":2},"answer":"12π"}</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Work from the annotated figure showing an annotated 3D solid. Based on the shown values, answer this question: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+Return a valid JSON object with key "answer".
+Answer rule: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"answer":"12π"}</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>{"evidence": {"MN": 9}, "answer": "324π"}</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>{"MN": 9}</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>pi_expression</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>measurement_ref_map</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>6467520649855215</v>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0017.png</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0017.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="288" customHeight="1">
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>task_geometry_analytical_3d_value</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>surface_area</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Look at the annotated image showing an annotated 3D solid. Read the marked measurements and answer: The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
+Return a valid JSON object with keys "evidence" and "answer" in that order.
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: EF, GH.
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"EF":2,"GH":3},"answer":8}</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Look at the annotated image showing an annotated 3D solid. Read the marked measurements and answer: The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
+Return a valid JSON object with key "answer".
+Answer: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>{"evidence": {"EF": 35, "GH": 49}, "answer": 4655}</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>{"EF": 35, "GH": 49}</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>measurement_ref_map</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>6563209679603169</v>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0010.png</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0010.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="288" customHeight="1">
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>task_geometry_analytical_3d_value</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>surface_area</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Use the image showing an annotated 3D solid. Question: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
+Return a valid JSON object with keys "evidence" and "answer" in that order.
+Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: ST, SU, TU, SV.
+Answer rule: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"ST":2,"SU":3,"TU":4,"SV":5},"answer":8}</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Use the image showing an annotated 3D solid. Question: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
+Return a valid JSON object with key "answer".
+Answer rule: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>{"evidence": {"ST": 15, "SU": 20, "TU": 25, "SV": 45}, "answer": 3000}</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>{"ST": 15, "SU": 20, "TU": 25, "SV": 45}</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>measurement_ref_map</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>6565138927499801</v>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0020.png</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0020.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="288" customHeight="1">
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>task_geometry_analytical_3d_value</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>surface_area</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>You are given an image showing an annotated 3D solid. Task: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
+Return a valid JSON object with keys "evidence" and "answer" in that order.
+Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: FG, FH, GH, FI.
+Answer format: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"FG":2,"FH":3,"GH":4,"FI":5},"answer":8}</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>You are given an image showing an annotated 3D solid. Task: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
+Return a valid JSON object with key "answer".
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>{"evidence": {"FG": 21, "FH": 28, "GH": 35, "FI": 42}, "answer": 4116}</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>{"FG": 21, "FH": 28, "GH": 35, "FI": 42}</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>measurement_ref_map</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>6600363319807691</v>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0011.png</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0011.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="288" customHeight="1">
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>task_geometry_analytical_3d_value</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>surface_area</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>The image shows an annotated 3D solid. The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
+Return a valid JSON object with keys "evidence" and "answer" in that order.
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: QR, ST.
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"QR":2,"ST":3},"answer":8}</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>The image shows an annotated 3D solid. The square pyramid has an annotated base side and slant height. What is its total surface area in square units?
+Return a valid JSON object with key "answer".
+Answer format: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>{"evidence": {"QR": 15, "ST": 42}, "answer": 1485}</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>{"QR": 15, "ST": 42}</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>measurement_ref_map</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>6788105196505530</v>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0016.png</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0016.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="288" customHeight="1">
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>task_geometry_analytical_3d_value</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>surface_area</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
+Return a valid JSON object with keys "evidence" and "answer" in that order.
+Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: HI, JI.
+Answer: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"HI":2,"JI":3},"answer":"12π"}</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
+Return a valid JSON object with key "answer".
+Answer: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"answer":"12π"}</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>{"evidence": {"HI": 27, "JI": 37}, "answer": "1728π"}</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>{"HI": 27, "JI": 37}</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>pi_expression</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>measurement_ref_map</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>6820722820145604</v>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0014.png</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0014.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="288" customHeight="1">
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>task_geometry_analytical_3d_value</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>surface_area</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Use the image showing an annotated 3D solid. Based on the shown values, answer this question: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+Return a valid JSON object with keys "evidence" and "answer" in that order.
+Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: YZ.
+Answer rule: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"YZ":2},"answer":"12π"}</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Use the image showing an annotated 3D solid. Based on the shown values, answer this question: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
+Return a valid JSON object with key "answer".
+Answer rule: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"answer":"12π"}</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>{"evidence": {"YZ": 5}, "answer": "100π"}</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>{"YZ": 5}</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>pi_expression</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>measurement_ref_map</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>7036686083602190</v>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0008.png</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0008.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="288" customHeight="1">
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>task_geometry_analytical_3d_value</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>surface_area</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Look at the annotated image showing an annotated 3D solid. Question: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
+Return a valid JSON object with keys "evidence" and "answer" in that order.
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: ST, TU, SV.
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"ST":2,"TU":3,"SV":4},"answer":8}</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Look at the annotated image showing an annotated 3D solid. Question: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
+Return a valid JSON object with key "answer".
+Answer format: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>{"evidence": {"ST": 49, "TU": 18, "SV": 40}, "answer": 7124}</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>{"ST": 49, "TU": 18, "SV": 40}</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>measurement_ref_map</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>7322459361145087</v>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0023.png</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0023.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="288" customHeight="1">
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>task_geometry_analytical_3d_value</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>surface_area</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Use the image showing an annotated 3D solid. The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
 Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: PQ, QR, PS.
 Answer: set "answer" to the value as an integer.
@@ -3869,622 +4445,46 @@
 {"evidence":{"PQ":2,"QR":3,"PS":4},"answer":8}</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
-Return a valid JSON object with key "answer".
-Answer rule: set "answer" to the value as an integer.
-Example JSON:
-{"answer":8}</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>{"evidence": {"PQ": 25, "QR": 20, "PS": 44}, "answer": 4960}</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>{"PQ": 25, "QR": 20, "PS": 44}</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>measurement_ref_map</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
-        <v>4525120154512047</v>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0001.png</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0001.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="288" customHeight="1">
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>task_geometry_analytical_3d_value</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>surface_area</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
-Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: ZA, BC.
-Answer format: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"ZA":2,"BC":3},"answer":"12π"}</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
-Return a valid JSON object with key "answer".
-Answer format: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>{"evidence": {"ZA": 10, "BC": 5}, "answer": "300π"}</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>{"ZA": 10, "BC": 5}</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>pi_expression</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>measurement_ref_map</t>
-        </is>
-      </c>
-      <c r="K16" t="n">
-        <v>4974663073616517</v>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0009.png</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0009.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="288" customHeight="1">
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>task_geometry_analytical_3d_value</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>surface_area</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>You are given an image showing an annotated 3D solid. Question: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
-Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: ZA, AB, ZC.
-Answer format: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"ZA":2,"AB":3,"ZC":4},"answer":8}</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>You are given an image showing an annotated 3D solid. Question: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
-Return a valid JSON object with key "answer".
-Answer rule: set "answer" to the value as an integer.
-Example JSON:
-{"answer":8}</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>{"evidence": {"ZA": 24, "AB": 36, "ZC": 48}, "answer": 7488}</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>{"ZA": 24, "AB": 36, "ZC": 48}</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>measurement_ref_map</t>
-        </is>
-      </c>
-      <c r="K17" t="n">
-        <v>6271914565665989</v>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0000.png</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0000.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="288" customHeight="1">
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>task_geometry_analytical_3d_value</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>surface_area</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
-Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: FG, HG.
-Answer requirement: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"FG":2,"HG":3},"answer":"12π"}</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
-Return a valid JSON object with key "answer".
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>{"evidence": {"FG": 5, "HG": 12}, "answer": "85π"}</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>{"FG": 5, "HG": 12}</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>pi_expression</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>measurement_ref_map</t>
-        </is>
-      </c>
-      <c r="K18" t="n">
-        <v>6573221049652373</v>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0007.png</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0007.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="288" customHeight="1">
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>task_geometry_analytical_3d_value</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>surface_area</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Look at the annotated image showing an annotated 3D solid. Task: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
-Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: PQ.
-Answer: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"PQ":2},"answer":"12π"}</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Look at the annotated image showing an annotated 3D solid. Task: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
-Return a valid JSON object with key "answer".
-Answer requirement: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>{"evidence": {"PQ": 7}, "answer": "196π"}</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>{"PQ": 7}</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>pi_expression</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>measurement_ref_map</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
-        <v>6579255519598814</v>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0006.png</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0006.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="288" customHeight="1">
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>task_geometry_analytical_3d_value</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>surface_area</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>The image shows an annotated 3D solid. Read the marked measurements and answer: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
-Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: GH, GI, HI, GJ.
-Answer: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"GH":2,"GI":3,"HI":4,"GJ":5},"answer":8}</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>The image shows an annotated 3D solid. Read the marked measurements and answer: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
-Return a valid JSON object with key "answer".
-Answer rule: set "answer" to the value as an integer.
-Example JSON:
-{"answer":8}</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>{"evidence": {"GH": 9, "GI": 12, "HI": 15, "GJ": 50}, "answer": 1908}</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>{"GH": 9, "GI": 12, "HI": 15, "GJ": 50}</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>measurement_ref_map</t>
-        </is>
-      </c>
-      <c r="K20" t="n">
-        <v>7035920139629747</v>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0018.png</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0018.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="288" customHeight="1">
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>task_geometry_analytical_3d_value</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>surface_area</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Look at the annotated image showing an annotated 3D solid. Question: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
-Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: MN, ON.
-Answer requirement: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"MN":2,"ON":3},"answer":"12π"}</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Look at the annotated image showing an annotated 3D solid. Question: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
-Return a valid JSON object with key "answer".
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>{"evidence": {"MN": 30, "ON": 33}, "answer": "1890π"}</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>{"MN": 30, "ON": 33}</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>pi_expression</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>measurement_ref_map</t>
-        </is>
-      </c>
-      <c r="K21" t="n">
-        <v>7049824546185202</v>
-      </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0004.png</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0004.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="288" customHeight="1">
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>task_geometry_analytical_3d_value</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>surface_area</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>The image shows an annotated 3D solid. Read the marked measurements and answer: The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
-Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: QR, ST.
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"QR":2,"ST":3},"answer":"12π"}</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>The image shows an annotated 3D solid. Read the marked measurements and answer: The cylinder has an annotated radius and height. What is its total surface area? Express the result in kπ form.
-Return a valid JSON object with key "answer".
-Answer: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>{"evidence": {"QR": 8, "ST": 30}, "answer": "608π"}</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>{"QR": 8, "ST": 30}</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>pi_expression</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>measurement_ref_map</t>
-        </is>
-      </c>
-      <c r="K22" t="n">
-        <v>7463300803331487</v>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0019.png</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0019.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="288" customHeight="1">
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>task_geometry_analytical_3d_value</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>surface_area</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
-Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: WX, XY, WZ.
-Answer requirement: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"WX":2,"XY":3,"WZ":4},"answer":8}</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Use the image showing an annotated 3D solid. The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the value as an integer.
 Example JSON:
 {"answer":8}</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>{"evidence": {"WX": 27, "XY": 5, "WZ": 37}, "answer": 2638}</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>{"WX": 27, "XY": 5, "WZ": 37}</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>{"evidence": {"PQ": 42, "QR": 35, "PS": 47}, "answer": 10178}</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>{"PQ": 42, "QR": 35, "PS": 47}</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>measurement_ref_map</t>
         </is>
       </c>
-      <c r="K23" t="n">
-        <v>7737344863052275</v>
-      </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0010.png</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="inlineStr">
-        <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0010.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="288" customHeight="1">
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>task_geometry_analytical_3d_value</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>surface_area</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Use the image showing an annotated 3D solid. Read the marked measurements and answer: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
-Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: XY, ZY.
-Answer: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"XY":2,"ZY":3},"answer":"12π"}</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Use the image showing an annotated 3D solid. Read the marked measurements and answer: The cone has an annotated radius and slant height. What is its total surface area? Express the result in kπ form.
-Return a valid JSON object with key "answer".
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>{"evidence": {"XY": 28, "ZY": 40}, "answer": "1904π"}</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>{"XY": 28, "ZY": 40}</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>pi_expression</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>measurement_ref_map</t>
-        </is>
-      </c>
       <c r="K24" t="n">
-        <v>7968173248390603</v>
+        <v>8075421881251309</v>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0014.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0005.png</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0014.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0005.json</t>
         </is>
       </c>
     </row>
@@ -4501,36 +4501,36 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Look at the annotated image showing an annotated 3D solid. Question: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
+          <t>Use the image showing an annotated 3D solid. Based on the shown values, answer this question: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: WX, WY, XY, WZ.
-Answer format: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"WX":2,"WY":3,"XY":4,"WZ":5},"answer":8}</t>
+Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: QR.
+Answer requirement: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"QR":2},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Look at the annotated image showing an annotated 3D solid. Question: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
+          <t>Use the image showing an annotated 3D solid. Based on the shown values, answer this question: The sphere has an annotated radius. What is its total surface area? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer rule: set "answer" to the value as an integer.
-Example JSON:
-{"answer":8}</t>
+Answer format: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"answer":"12π"}</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"WX": 12, "WY": 16, "XY": 20, "WZ": 22}, "answer": 1248}</t>
+          <t>{"evidence": {"QR": 20}, "answer": "1600π"}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>{"WX": 12, "WY": 16, "XY": 20, "WZ": 22}</t>
+          <t>{"QR": 20}</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>pi_expression</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -4539,16 +4539,16 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>8873944668682965</v>
+        <v>8215287962366592</v>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0021.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0022.png</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0021.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0022.json</t>
         </is>
       </c>
     </row>
@@ -4565,17 +4565,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Read the marked measurements and answer: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
+          <t>Work from the annotated figure showing an annotated 3D solid. Task: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: VW, VX, WX, VY.
-Answer: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"VW":2,"VX":3,"WX":4,"VY":5},"answer":8}</t>
+Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: GH, HI, GJ.
+Answer format: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"GH":2,"HI":3,"GJ":4},"answer":8}</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Read the marked measurements and answer: The triangular prism has annotated side lengths for the triangular base and an annotated prism length. What is its total surface area in square units?
+          <t>Work from the annotated figure showing an annotated 3D solid. Task: The rectangular prism has annotated length, width, and height. What is its total surface area in square units?
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the value as an integer.
 Example JSON:
@@ -4584,12 +4584,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"VW": 9, "VX": 40, "WX": 41, "VY": 37}, "answer": 3690}</t>
+          <t>{"evidence": {"GH": 26, "HI": 13, "GJ": 49}, "answer": 4498}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>{"VW": 9, "VX": 40, "WX": 41, "VY": 37}</t>
+          <t>{"GH": 26, "HI": 13, "GJ": 49}</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -4603,16 +4603,16 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>8896945692663174</v>
+        <v>8516970128904864</v>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0011.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/surface_area/0009.png</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0011.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/surface_area/0009.json</t>
         </is>
       </c>
     </row>
@@ -4726,36 +4726,36 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. Task: The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Read the marked measurements and answer: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: WX, YZ.
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"WX":2,"YZ":3},"answer":"12π"}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: FG, FH, FI.
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"FG":2,"FH":3,"FI":4},"answer":8}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. Task: The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Read the marked measurements and answer: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer field: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer format: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"WX": 18, "YZ": 35}, "answer": "11340π"}</t>
+          <t>{"evidence": {"FG": 10, "FH": 23, "FI": 15}, "answer": 1725}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>{"WX": 18, "YZ": 35}</t>
+          <t>{"FG": 10, "FH": 23, "FI": 15}</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -4764,16 +4764,16 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>212728511500442</v>
+        <v>87139262147013</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0014.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0013.png</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0014.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0013.json</t>
         </is>
       </c>
     </row>
@@ -4790,36 +4790,36 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Read the marked measurements and answer: The cone has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Use the image showing an annotated 3D solid. Question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: WX, YW.
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"WX":2,"YW":3},"answer":"12π"}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: EF, FG, EH.
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"EF":2,"FG":3,"EH":4},"answer":8}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Read the marked measurements and answer: The cone has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Use the image showing an annotated 3D solid. Question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer field: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer requirement: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"WX": 47, "YW": 27}, "answer": "19881π"}</t>
+          <t>{"evidence": {"EF": 47, "FG": 41, "EH": 17}, "answer": 32759}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>{"WX": 47, "YW": 27}</t>
+          <t>{"EF": 47, "FG": 41, "EH": 17}</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -4828,16 +4828,16 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>552340278203500</v>
+        <v>558792218275212</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0023.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0020.png</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0023.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0020.json</t>
         </is>
       </c>
     </row>
@@ -4854,36 +4854,36 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Based on the shown values, answer this question: The sphere has an annotated radius. What is its volume? Express the result in kπ form.
+          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: UV.
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"UV":2},"answer":"12π"}</t>
+Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: ZA, ZB, ZC.
+Answer format: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"ZA":2,"ZB":3,"ZC":4},"answer":8}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Based on the shown values, answer this question: The sphere has an annotated radius. What is its volume? Express the result in kπ form.
+          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer format: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer format: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"UV": 6}, "answer": "288π"}</t>
+          <t>{"evidence": {"ZA": 50, "ZB": 21, "ZC": 7}, "answer": 3675}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>{"UV": 6}</t>
+          <t>{"ZA": 50, "ZB": 21, "ZC": 7}</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -4892,16 +4892,16 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>864403571948945</v>
+        <v>576512490849321</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0005.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0015.png</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0005.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0015.json</t>
         </is>
       </c>
     </row>
@@ -4918,36 +4918,36 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. The sphere has an annotated radius. What is its volume? Express the result in kπ form.
+          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: WX.
-Answer format: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"WX":2},"answer":"12π"}</t>
+Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: IJ, JK, IL.
+Answer rule: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"IJ":2,"JK":3,"IL":4},"answer":8}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. The sphere has an annotated radius. What is its volume? Express the result in kπ form.
+          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"WX": 6}, "answer": "288π"}</t>
+          <t>{"evidence": {"IJ": 22, "JK": 40, "IL": 8}, "answer": 7040}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>{"WX": 6}</t>
+          <t>{"IJ": 22, "JK": 40, "IL": 8}</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -4956,16 +4956,16 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>901534776250193</v>
+        <v>1105853822194894</v>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0008.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0007.png</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0008.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0007.json</t>
         </is>
       </c>
     </row>
@@ -4982,31 +4982,31 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Read the marked measurements and answer: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
+          <t>The image shows an annotated 3D solid. Question: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: YZ, YA, YB.
-Answer format: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"YZ":2,"YA":3,"YB":4},"answer":8}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: XY, ZA.
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"XY":2,"ZA":3},"answer":8}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Read the marked measurements and answer: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
+          <t>The image shows an annotated 3D solid. Question: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer format: set "answer" to the value as an integer.
+Answer field: set "answer" to the value as an integer.
 Example JSON:
 {"answer":8}</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"YZ": 7, "YA": 38, "YB": 38}, "answer": 5054}</t>
+          <t>{"evidence": {"XY": 33, "ZA": 30}, "answer": 10890}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>{"YZ": 7, "YA": 38, "YB": 38}</t>
+          <t>{"XY": 33, "ZA": 30}</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -5020,16 +5020,16 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>941863908481627</v>
+        <v>1118229189304009</v>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0021.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0002.png</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0021.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0002.json</t>
         </is>
       </c>
     </row>
@@ -5046,31 +5046,31 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Task: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
+          <t>Use the image showing an annotated 3D solid. The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: AB, AC, AD.
-Answer requirement: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"AB":2,"AC":3,"AD":4},"answer":8}</t>
+Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: RS, RT, RU.
+Answer format: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"RS":2,"RT":3,"RU":4},"answer":8}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Task: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
+          <t>Use the image showing an annotated 3D solid. The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer field: set "answer" to the value as an integer.
+Answer format: set "answer" to the value as an integer.
 Example JSON:
 {"answer":8}</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"AB": 48, "AC": 37, "AD": 48}, "answer": 42624}</t>
+          <t>{"evidence": {"RS": 25, "RT": 42, "RU": 40}, "answer": 21000}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>{"AB": 48, "AC": 37, "AD": 48}</t>
+          <t>{"RS": 25, "RT": 42, "RU": 40}</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -5084,16 +5084,16 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>1125398503401974</v>
+        <v>1704617513677448</v>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0009.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0022.png</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0009.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0022.json</t>
         </is>
       </c>
     </row>
@@ -5110,36 +5110,36 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Task: The cone has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Based on the shown values, answer this question: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: RS, TR.
-Answer requirement: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"RS":2,"TR":3},"answer":"12π"}</t>
+Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: QR, QS, QT.
+Answer format: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"QR":2,"QS":3,"QT":4},"answer":8}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Task: The cone has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Based on the shown values, answer this question: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer field: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer requirement: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"RS": 9, "TR": 41}, "answer": "1107π"}</t>
+          <t>{"evidence": {"QR": 22, "QS": 28, "QT": 11}, "answer": 3388}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>{"RS": 9, "TR": 41}</t>
+          <t>{"QR": 22, "QS": 28, "QT": 11}</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -5148,16 +5148,16 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1223829043012499</v>
+        <v>1979267592240054</v>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0010.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0011.png</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0010.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0011.json</t>
         </is>
       </c>
     </row>
@@ -5174,36 +5174,36 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
+          <t>Work from the annotated figure showing an annotated 3D solid. Task: The sphere has an annotated radius. What is its volume? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: MN, MO, MP.
-Answer format: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"MN":2,"MO":3,"MP":4},"answer":8}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: HI.
+Answer field: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"HI":2},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
+          <t>Work from the annotated figure showing an annotated 3D solid. Task: The sphere has an annotated radius. What is its volume? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer format: set "answer" to the value as an integer.
-Example JSON:
-{"answer":8}</t>
+Answer requirement: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"answer":"12π"}</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"MN": 16, "MO": 27, "MP": 36}, "answer": 7776}</t>
+          <t>{"evidence": {"HI": 18}, "answer": "7776π"}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>{"MN": 16, "MO": 27, "MP": 36}</t>
+          <t>{"HI": 18}</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>pi_expression</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -5212,16 +5212,16 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>1583227017386269</v>
+        <v>2611919943941541</v>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0019.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0016.png</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0019.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0016.json</t>
         </is>
       </c>
     </row>
@@ -5238,36 +5238,36 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>You are given an image showing an annotated 3D solid. Question: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: JK, LM.
-Answer format: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"JK":2,"LM":3},"answer":"12π"}</t>
+Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: VW, VX, VY.
+Answer requirement: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"VW":2,"VX":3,"VY":4},"answer":8}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>You are given an image showing an annotated 3D solid. Question: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer field: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"JK": 44, "LM": 11}, "answer": "21296π"}</t>
+          <t>{"evidence": {"VW": 10, "VX": 18, "VY": 10}, "answer": 900}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>{"JK": 44, "LM": 11}</t>
+          <t>{"VW": 10, "VX": 18, "VY": 10}</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -5276,16 +5276,16 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>1936806105130654</v>
+        <v>2829994374986399</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0024.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0008.png</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0024.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0008.json</t>
         </is>
       </c>
     </row>
@@ -5302,31 +5302,31 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Look at the annotated image showing an annotated 3D solid. The cone has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Question: The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: KL, MK.
+Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: EF, GH.
 Answer rule: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
-{"evidence":{"KL":2,"MK":3},"answer":"12π"}</t>
+{"evidence":{"EF":2,"GH":3},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Look at the annotated image showing an annotated 3D solid. The cone has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Question: The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
+Answer format: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
 {"answer":"12π"}</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"KL": 42, "MK": 5}, "answer": "2940π"}</t>
+          <t>{"evidence": {"EF": 40, "GH": 23}, "answer": "36800π"}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>{"KL": 42, "MK": 5}</t>
+          <t>{"EF": 40, "GH": 23}</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -5340,16 +5340,16 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>1992575116286964</v>
+        <v>2897426442381988</v>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0000.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0019.png</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0000.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0019.json</t>
         </is>
       </c>
     </row>
@@ -5366,36 +5366,36 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Read the marked measurements and answer: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
+          <t>Look at the annotated image showing an annotated 3D solid. Task: The cone has an annotated radius and height. What is its volume? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: HI, JK.
-Answer format: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"HI":2,"JK":3},"answer":8}</t>
+Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: YZ, AY.
+Answer requirement: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"YZ":2,"AY":3},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Read the marked measurements and answer: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
+          <t>Look at the annotated image showing an annotated 3D solid. Task: The cone has an annotated radius and height. What is its volume? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer field: set "answer" to the value as an integer.
-Example JSON:
-{"answer":8}</t>
+Answer format: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"answer":"12π"}</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"HI": 33, "JK": 32}, "answer": 11616}</t>
+          <t>{"evidence": {"YZ": 34, "AY": 24}, "answer": "9248π"}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>{"HI": 33, "JK": 32}</t>
+          <t>{"YZ": 34, "AY": 24}</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>pi_expression</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -5404,16 +5404,16 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>2248381729004976</v>
+        <v>3176063686641968</v>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0015.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0018.png</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0015.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0018.json</t>
         </is>
       </c>
     </row>
@@ -5430,36 +5430,36 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>You are given an image showing an annotated 3D solid. The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: DE, FG.
-Answer format: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"DE":2,"FG":3},"answer":"12π"}</t>
+Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: EF, GH.
+Answer requirement: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"EF":2,"GH":3},"answer":8}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>You are given an image showing an annotated 3D solid. The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer format: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"DE": 27, "FG": 10}, "answer": "7290π"}</t>
+          <t>{"evidence": {"EF": 27, "GH": 10}, "answer": 2430}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>{"DE": 27, "FG": 10}</t>
+          <t>{"EF": 27, "GH": 10}</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -5468,16 +5468,16 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>2467830548565600</v>
+        <v>3453265177121059</v>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0011.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0021.png</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0011.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0021.json</t>
         </is>
       </c>
     </row>
@@ -5494,36 +5494,36 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Question: The sphere has an annotated radius. What is its volume? Express the result in kπ form.
+          <t>Look at the annotated image showing an annotated 3D solid. The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: ZA.
-Answer format: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"ZA":2},"answer":"12π"}</t>
+Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: XY, XZ, XA.
+Answer rule: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"XY":2,"XZ":3,"XA":4},"answer":8}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Question: The sphere has an annotated radius. What is its volume? Express the result in kπ form.
+          <t>Look at the annotated image showing an annotated 3D solid. The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"ZA": 30}, "answer": "36000π"}</t>
+          <t>{"evidence": {"XY": 5, "XZ": 42, "XA": 36}, "answer": 3780}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>{"ZA": 30}</t>
+          <t>{"XY": 5, "XZ": 42, "XA": 36}</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -5532,16 +5532,16 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2988666460797354</v>
+        <v>4208138728157935</v>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0020.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0023.png</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0020.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0023.json</t>
         </is>
       </c>
     </row>
@@ -5558,31 +5558,31 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
+          <t>Work from the annotated figure showing an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: XY, YZ, XA.
+Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: DE, EF, DG.
 Answer rule: set "answer" to the value as an integer.
 Example JSON:
-{"evidence":{"XY":2,"YZ":3,"XA":4},"answer":8}</t>
+{"evidence":{"DE":2,"EF":3,"DG":4},"answer":8}</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
+          <t>Work from the annotated figure showing an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer format: set "answer" to the value as an integer.
+Answer field: set "answer" to the value as an integer.
 Example JSON:
 {"answer":8}</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"XY": 23, "YZ": 32, "XA": 13}, "answer": 9568}</t>
+          <t>{"evidence": {"DE": 23, "EF": 8, "DG": 15}, "answer": 2760}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>{"XY": 23, "YZ": 32, "XA": 13}</t>
+          <t>{"DE": 23, "EF": 8, "DG": 15}</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -5596,16 +5596,16 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>3318912934090459</v>
+        <v>4276514804363001</v>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0004.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0012.png</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0004.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0012.json</t>
         </is>
       </c>
     </row>
@@ -5622,36 +5622,36 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. Task: The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Read the marked measurements and answer: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: VW, XY.
-Answer format: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"VW":2,"XY":3},"answer":"12π"}</t>
+Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: OP, OQ, OR.
+Answer rule: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"OP":2,"OQ":3,"OR":4},"answer":8}</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. Task: The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Read the marked measurements and answer: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"VW": 36, "XY": 28}, "answer": "36288π"}</t>
+          <t>{"evidence": {"OP": 16, "OQ": 26, "OR": 40}, "answer": 8320}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>{"VW": 36, "XY": 28}</t>
+          <t>{"OP": 16, "OQ": 26, "OR": 40}</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -5660,16 +5660,16 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>4398992449688888</v>
+        <v>4821582613905229</v>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0012.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0003.png</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0012.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0003.json</t>
         </is>
       </c>
     </row>
@@ -5686,36 +5686,36 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Task: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
+          <t>Use the image showing an annotated 3D solid. Task: The sphere has an annotated radius. What is its volume? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: YZ, ZA, YB.
-Answer format: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"YZ":2,"ZA":3,"YB":4},"answer":8}</t>
+Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: VW.
+Answer: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"VW":2},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Task: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
+          <t>Use the image showing an annotated 3D solid. Task: The sphere has an annotated radius. What is its volume? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer: set "answer" to the value as an integer.
-Example JSON:
-{"answer":8}</t>
+Answer requirement: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"answer":"12π"}</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"YZ": 43, "ZA": 29, "YB": 18}, "answer": 22446}</t>
+          <t>{"evidence": {"VW": 48}, "answer": "147456π"}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>{"YZ": 43, "ZA": 29, "YB": 18}</t>
+          <t>{"VW": 48}</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>pi_expression</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -5724,16 +5724,16 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>4469300212369752</v>
+        <v>5053364104794416</v>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0003.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0005.png</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0003.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0005.json</t>
         </is>
       </c>
     </row>
@@ -5750,36 +5750,36 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Task: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
+          <t>Work from the annotated figure showing an annotated 3D solid. Task: The cone has an annotated radius and height. What is its volume? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: UV, UW, UX.
-Answer format: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"UV":2,"UW":3,"UX":4},"answer":8}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: JK, LJ.
+Answer field: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"JK":2,"LJ":3},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Task: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
+          <t>Work from the annotated figure showing an annotated 3D solid. Task: The cone has an annotated radius and height. What is its volume? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer field: set "answer" to the value as an integer.
-Example JSON:
-{"answer":8}</t>
+Answer: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"answer":"12π"}</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"UV": 36, "UW": 6, "UX": 11}, "answer": 1188}</t>
+          <t>{"evidence": {"JK": 39, "LJ": 33}, "answer": "16731π"}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>{"UV": 36, "UW": 6, "UX": 11}</t>
+          <t>{"JK": 39, "LJ": 33}</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>pi_expression</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -5788,16 +5788,16 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>4628280926046570</v>
+        <v>5689253998843440</v>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0006.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0014.png</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0006.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0014.json</t>
         </is>
       </c>
     </row>
@@ -5814,31 +5814,31 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>You are given an image showing an annotated 3D solid. Task: The sphere has an annotated radius. What is its volume? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: UV, WX.
+Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: AB.
 Answer: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
-{"evidence":{"UV":2,"WX":3},"answer":"12π"}</t>
+{"evidence":{"AB":2},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>You are given an image showing an annotated 3D solid. Task: The sphere has an annotated radius. What is its volume? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer requirement: set "answer" to the value in the form kπ (for example 12π).
+Answer rule: set "answer" to the value in the form kπ (for example 12π).
 Example JSON:
 {"answer":"12π"}</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"UV": 21, "WX": 50}, "answer": "22050π"}</t>
+          <t>{"evidence": {"AB": 24}, "answer": "18432π"}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>{"UV": 21, "WX": 50}</t>
+          <t>{"AB": 24}</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -5852,16 +5852,16 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>4857182651944177</v>
+        <v>5964740903880011</v>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0017.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0001.png</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0017.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0001.json</t>
         </is>
       </c>
     </row>
@@ -5878,36 +5878,36 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: TU, VW.
-Answer requirement: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"TU":2,"VW":3},"answer":"12π"}</t>
+Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: OP, OQ, OR.
+Answer rule: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"OP":2,"OQ":3,"OR":4},"answer":8}</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Work from the annotated figure showing an annotated 3D solid. The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer field: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer rule: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"TU": 10, "VW": 28}, "answer": "2800π"}</t>
+          <t>{"evidence": {"OP": 39, "OQ": 8, "OR": 29}, "answer": 4524}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>{"TU": 10, "VW": 28}</t>
+          <t>{"OP": 39, "OQ": 8, "OR": 29}</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -5916,16 +5916,16 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>6065155439809233</v>
+        <v>6102506914741584</v>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0002.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0010.png</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0002.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0010.json</t>
         </is>
       </c>
     </row>
@@ -5942,31 +5942,31 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Task: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
+          <t>The image shows an annotated 3D solid. Task: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: OP, QR.
-Answer: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"OP":2,"QR":3},"answer":8}</t>
+Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: DE, FG.
+Answer rule: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"DE":2,"FG":3},"answer":8}</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Use the image showing an annotated 3D solid. Task: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
+          <t>The image shows an annotated 3D solid. Task: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer requirement: set "answer" to the value as an integer.
+Answer rule: set "answer" to the value as an integer.
 Example JSON:
 {"answer":8}</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"OP": 10, "QR": 15}, "answer": 500}</t>
+          <t>{"evidence": {"DE": 27, "FG": 19}, "answer": 4617}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>{"OP": 10, "QR": 15}</t>
+          <t>{"DE": 27, "FG": 19}</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -5980,16 +5980,16 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>6154562800781828</v>
+        <v>6308953695344084</v>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0013.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0024.png</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0013.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0024.json</t>
         </is>
       </c>
     </row>
@@ -6006,36 +6006,36 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The cone has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Task: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: ZA, BZ.
-Answer rule: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"evidence":{"ZA":2,"BZ":3},"answer":"12π"}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: VW, VX, VY.
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"VW":2,"VX":3,"VY":4},"answer":8}</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The cone has an annotated radius and height. What is its volume? Express the result in kπ form.
+          <t>Work from the annotated figure showing an annotated 3D solid. Task: The triangular prism has an annotated triangle base, triangle height, and prism length. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer field: set "answer" to the value in the form kπ (for example 12π).
-Example JSON:
-{"answer":"12π"}</t>
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"answer":8}</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"ZA": 36, "BZ": 43}, "answer": "18576π"}</t>
+          <t>{"evidence": {"VW": 36, "VX": 41, "VY": 25}, "answer": 18450}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>{"ZA": 36, "BZ": 43}</t>
+          <t>{"VW": 36, "VX": 41, "VY": 25}</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>pi_expression</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -6044,16 +6044,16 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>6668224475224908</v>
+        <v>6513527728746925</v>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0001.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0017.png</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0001.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0017.json</t>
         </is>
       </c>
     </row>
@@ -6070,36 +6070,36 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
+          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: PQ, QR, PS.
-Answer: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"PQ":2,"QR":3,"PS":4},"answer":8}</t>
+Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: HI, JK.
+Answer: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"HI":2,"JK":3},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>You are given an image showing an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
+          <t>You are given an image showing an annotated 3D solid. Read the marked measurements and answer: The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer format: set "answer" to the value as an integer.
-Example JSON:
-{"answer":8}</t>
+Answer: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"answer":"12π"}</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"PQ": 11, "QR": 13, "PS": 24}, "answer": 3432}</t>
+          <t>{"evidence": {"HI": 32, "JK": 39}, "answer": "39936π"}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>{"PQ": 11, "QR": 13, "PS": 24}</t>
+          <t>{"HI": 32, "JK": 39}</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>pi_expression</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -6108,16 +6108,16 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>7278171396682207</v>
+        <v>7027638525325108</v>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0022.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0006.png</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0022.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0006.json</t>
         </is>
       </c>
     </row>
@@ -6134,36 +6134,36 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
+          <t>Use the image showing an annotated 3D solid. The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: XY, YZ, XA.
-Answer format: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"XY":2,"YZ":3,"XA":4},"answer":8}</t>
+Evidence rule: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: OP, QR.
+Answer rule: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"evidence":{"OP":2,"QR":3},"answer":"12π"}</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
+          <t>Use the image showing an annotated 3D solid. The cylinder has an annotated radius and height. What is its volume? Express the result in kπ form.
 Return a valid JSON object with key "answer".
-Answer field: set "answer" to the value as an integer.
-Example JSON:
-{"answer":8}</t>
+Answer format: set "answer" to the value in the form kπ (for example 12π).
+Example JSON:
+{"answer":"12π"}</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"XY": 38, "YZ": 50, "XA": 10}, "answer": 19000}</t>
+          <t>{"evidence": {"OP": 17, "QR": 22}, "answer": "6358π"}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>{"XY": 38, "YZ": 50, "XA": 10}</t>
+          <t>{"OP": 17, "QR": 22}</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>pi_expression</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -6172,16 +6172,16 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>7977760448128855</v>
+        <v>7081169466265394</v>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0018.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0004.png</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0018.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0004.json</t>
         </is>
       </c>
     </row>
@@ -6198,31 +6198,31 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Question: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
+          <t>Work from the annotated figure showing an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: AB, CD.
-Answer requirement: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"AB":2,"CD":3},"answer":8}</t>
+Evidence requirement: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: LM, MN, LO.
+Answer format: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"LM":2,"MN":3,"LO":4},"answer":8}</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>The image shows an annotated 3D solid. Question: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
+          <t>Work from the annotated figure showing an annotated 3D solid. Based on the shown values, answer this question: The rectangular prism has annotated length, width, and height. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer format: set "answer" to the value as an integer.
+Answer: set "answer" to the value as an integer.
 Example JSON:
 {"answer":8}</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"AB": 34, "CD": 15}, "answer": 5780}</t>
+          <t>{"evidence": {"LM": 6, "MN": 50, "LO": 36}, "answer": 10800}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>{"AB": 34, "CD": 15}</t>
+          <t>{"LM": 6, "MN": 50, "LO": 36}</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -6236,16 +6236,16 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>8524643456606325</v>
+        <v>7252074147112353</v>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0007.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0000.png</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0007.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0000.json</t>
         </is>
       </c>
     </row>
@@ -6262,31 +6262,31 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Look at the annotated image showing an annotated 3D solid. Read the marked measurements and answer: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
+          <t>You are given an image showing an annotated 3D solid. Task: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: XY, ZA.
-Answer: set "answer" to the value as an integer.
-Example JSON:
-{"evidence":{"XY":2,"ZA":3},"answer":8}</t>
+Evidence field: set "evidence" to a JSON object that maps each required annotation label to its shown measurement value. Required annotations: YZ, AB.
+Answer field: set "answer" to the value as an integer.
+Example JSON:
+{"evidence":{"YZ":2,"AB":3},"answer":8}</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Look at the annotated image showing an annotated 3D solid. Read the marked measurements and answer: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
+          <t>You are given an image showing an annotated 3D solid. Task: The square pyramid has an annotated base side and vertical height. What is its volume in cubic units?
 Return a valid JSON object with key "answer".
-Answer field: set "answer" to the value as an integer.
+Answer rule: set "answer" to the value as an integer.
 Example JSON:
 {"answer":8}</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": {"XY": 6, "ZA": 23}, "answer": 276}</t>
+          <t>{"evidence": {"YZ": 27, "AB": 50}, "answer": 12150}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>{"XY": 6, "ZA": 23}</t>
+          <t>{"YZ": 27, "AB": 50}</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -6300,16 +6300,16 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>8844038502752275</v>
+        <v>7418239730482128</v>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/images/volume/0016.png</t>
+          <t>geometry/task_geometry_analytical_3d_value/images/volume/0009.png</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>geometry/task_geometry_analytical_3d_value/data/volume/0016.json</t>
+          <t>geometry/task_geometry_analytical_3d_value/data/volume/0009.json</t>
         </is>
       </c>
     </row>

</xml_diff>